<commit_message>
Add Jan/Feb/Apr invoice rows to 견적 sheet
Add 260113, 260211, 260409 events from InterMD invoices to the 견적
sheet, sorted chronologically with the existing June events.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pUtUgEDNCUwkbRtZ83UEP
</commit_message>
<xml_diff>
--- a/2026_GI_견적_260514_update.xlsx
+++ b/2026_GI_견적_260514_update.xlsx
@@ -1152,7 +1152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1198,7 +1198,7 @@
     <row r="2">
       <c r="A2" s="70" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-01-13</t>
         </is>
       </c>
       <c r="B2" s="70" t="inlineStr">
@@ -1208,23 +1208,23 @@
       </c>
       <c r="C2" s="70" t="inlineStr">
         <is>
-          <t>NOW STRIDE SYMPOSIUM</t>
+          <t>담소 심포지엄 웨비나</t>
         </is>
       </c>
       <c r="D2" s="71" t="n">
         <v>5250000</v>
       </c>
       <c r="E2" s="71" t="n">
-        <v>2900000</v>
+        <v>5015000</v>
       </c>
       <c r="F2" s="72" t="n">
-        <v>8150000</v>
+        <v>10265000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="70" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="B3" s="70" t="inlineStr">
@@ -1241,16 +1241,16 @@
         <v>5250000</v>
       </c>
       <c r="E3" s="71" t="n">
-        <v>3750000</v>
+        <v>3860000</v>
       </c>
       <c r="F3" s="72" t="n">
-        <v>9000000</v>
+        <v>9110000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="70" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-04-09</t>
         </is>
       </c>
       <c r="B4" s="70" t="inlineStr">
@@ -1260,23 +1260,23 @@
       </c>
       <c r="C4" s="70" t="inlineStr">
         <is>
-          <t>HIT SYMPOSIUM Webinar</t>
+          <t>간담명료 웨비나 심포지엄</t>
         </is>
       </c>
       <c r="D4" s="71" t="n">
         <v>5250000</v>
       </c>
       <c r="E4" s="71" t="n">
-        <v>2078000</v>
+        <v>2331000</v>
       </c>
       <c r="F4" s="72" t="n">
-        <v>7328000</v>
+        <v>7581000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="70" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B5" s="70" t="inlineStr">
@@ -1293,14 +1293,92 @@
         <v>5250000</v>
       </c>
       <c r="E5" s="71" t="n">
+        <v>2900000</v>
+      </c>
+      <c r="F5" s="72" t="n">
+        <v>8150000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="70" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B6" s="70" t="inlineStr">
+        <is>
+          <t>임핀지</t>
+        </is>
+      </c>
+      <c r="C6" s="70" t="inlineStr">
+        <is>
+          <t>간담명료 웨비나 심포지엄</t>
+        </is>
+      </c>
+      <c r="D6" s="71" t="n">
+        <v>5250000</v>
+      </c>
+      <c r="E6" s="71" t="n">
+        <v>3750000</v>
+      </c>
+      <c r="F6" s="72" t="n">
+        <v>9000000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="70" t="inlineStr">
+        <is>
+          <t>2026-06-15</t>
+        </is>
+      </c>
+      <c r="B7" s="70" t="inlineStr">
+        <is>
+          <t>임핀지</t>
+        </is>
+      </c>
+      <c r="C7" s="70" t="inlineStr">
+        <is>
+          <t>HIT SYMPOSIUM Webinar</t>
+        </is>
+      </c>
+      <c r="D7" s="71" t="n">
+        <v>5250000</v>
+      </c>
+      <c r="E7" s="71" t="n">
+        <v>2078000</v>
+      </c>
+      <c r="F7" s="72" t="n">
+        <v>7328000</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="70" t="inlineStr">
+        <is>
+          <t>2026-06-17</t>
+        </is>
+      </c>
+      <c r="B8" s="70" t="inlineStr">
+        <is>
+          <t>임핀지</t>
+        </is>
+      </c>
+      <c r="C8" s="70" t="inlineStr">
+        <is>
+          <t>NOW STRIDE SYMPOSIUM</t>
+        </is>
+      </c>
+      <c r="D8" s="71" t="n">
+        <v>5250000</v>
+      </c>
+      <c r="E8" s="71" t="n">
         <v>1000000</v>
       </c>
-      <c r="F5" s="72" t="n">
+      <c r="F8" s="72" t="n">
         <v>6250000</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="73" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="73" t="inlineStr">
         <is>
           <t>※VAT 별도</t>
         </is>

</xml_diff>

<commit_message>
Add 6/23 Imfinzi Web Symposium row to 견적 sheet
Add 260623 (부산 윈덤 그랜드) event from InterMD quotation:
기본단가 5,250,000 + 추가비용 2,700,000 = 7,950,000.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016pUtUgEDNCUwkbRtZ83UEP
</commit_message>
<xml_diff>
--- a/2026_GI_견적_260514_update.xlsx
+++ b/2026_GI_견적_260514_update.xlsx
@@ -1152,7 +1152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1378,7 +1378,33 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="73" t="inlineStr">
+      <c r="A9" s="70" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>임핀지</t>
+        </is>
+      </c>
+      <c r="C9" s="70" t="inlineStr">
+        <is>
+          <t>간담명료 web SYMPOSIUM</t>
+        </is>
+      </c>
+      <c r="D9" s="71" t="n">
+        <v>5250000</v>
+      </c>
+      <c r="E9" s="71" t="n">
+        <v>2700000</v>
+      </c>
+      <c r="F9" s="72" t="n">
+        <v>7950000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="73" t="inlineStr">
         <is>
           <t>※VAT 별도</t>
         </is>

</xml_diff>